<commit_message>
feat: unmatched invoices sending
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -4314,64 +4314,184 @@
       </c>
     </row>
     <row r="94" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="7"/>
-      <c r="B94" s="6"/>
-      <c r="C94" s="6"/>
-      <c r="D94" s="6"/>
-      <c r="E94" s="6"/>
-      <c r="F94" s="6"/>
-      <c r="G94" s="6"/>
-      <c r="H94" s="6"/>
-      <c r="I94" s="6"/>
-      <c r="J94" s="11"/>
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>VJA2627025509</t>
+        </is>
+      </c>
+      <c r="B94" s="4">
+        <v>46191</v>
+      </c>
+      <c r="C94" s="5"/>
+      <c r="D94" s="5">
+        <v>64837</v>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>TAPDIYA HOME DECOR</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>TAPDIYA HOME DECOR</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>AURANGABAD</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>BATCO TPT</t>
+        </is>
+      </c>
+      <c r="I94" s="5"/>
+      <c r="J94" s="9"/>
     </row>
     <row r="95" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="7"/>
-      <c r="B95" s="6"/>
-      <c r="C95" s="6"/>
-      <c r="D95" s="6"/>
-      <c r="E95" s="6"/>
-      <c r="F95" s="6"/>
-      <c r="G95" s="6"/>
-      <c r="H95" s="6"/>
-      <c r="I95" s="6"/>
-      <c r="J95" s="11"/>
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>VJA2627025521</t>
+        </is>
+      </c>
+      <c r="B95" s="4">
+        <v>46191</v>
+      </c>
+      <c r="C95" s="5"/>
+      <c r="D95" s="5">
+        <v>64866</v>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>MD COLLECTION</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>MD COLLECTION</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>SURAT</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>R R TRANSPORT</t>
+        </is>
+      </c>
+      <c r="I95" s="5"/>
+      <c r="J95" s="9"/>
     </row>
     <row r="96" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="7"/>
-      <c r="B96" s="6"/>
-      <c r="C96" s="6"/>
-      <c r="D96" s="6"/>
-      <c r="E96" s="6"/>
-      <c r="F96" s="6"/>
-      <c r="G96" s="6"/>
-      <c r="H96" s="6"/>
-      <c r="I96" s="6"/>
-      <c r="J96" s="11"/>
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>VJA2627026079</t>
+        </is>
+      </c>
+      <c r="B96" s="4">
+        <v>46192</v>
+      </c>
+      <c r="C96" s="5"/>
+      <c r="D96" s="5">
+        <v>66388</v>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>R.K. ENTERPRISE ADV</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>R.K. ENTERPRISE</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>CUTTACK</t>
+        </is>
+      </c>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>BALAJI LOGISTICS</t>
+        </is>
+      </c>
+      <c r="I96" s="5"/>
+      <c r="J96" s="9"/>
     </row>
     <row r="97" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="7"/>
-      <c r="B97" s="6"/>
-      <c r="C97" s="6"/>
-      <c r="D97" s="6"/>
-      <c r="E97" s="6"/>
-      <c r="F97" s="6"/>
-      <c r="G97" s="6"/>
-      <c r="H97" s="6"/>
-      <c r="I97" s="6"/>
-      <c r="J97" s="11"/>
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>VJA2627026365</t>
+        </is>
+      </c>
+      <c r="B97" s="4">
+        <v>46193</v>
+      </c>
+      <c r="C97" s="5"/>
+      <c r="D97" s="5">
+        <v>67105</v>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>SIDDHARTH (  VADODARA )</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>SIDDHARTH (  Vadodara )</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>VADODARA</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>KABRA EXPRESS</t>
+        </is>
+      </c>
+      <c r="I97" s="5"/>
+      <c r="J97" s="9"/>
     </row>
     <row r="98" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="7"/>
-      <c r="B98" s="6"/>
-      <c r="C98" s="6"/>
-      <c r="D98" s="6"/>
-      <c r="E98" s="6"/>
-      <c r="F98" s="6"/>
-      <c r="G98" s="6"/>
-      <c r="H98" s="6"/>
-      <c r="I98" s="6"/>
-      <c r="J98" s="11"/>
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>VJA2627026376</t>
+        </is>
+      </c>
+      <c r="B98" s="4">
+        <v>46193</v>
+      </c>
+      <c r="C98" s="5"/>
+      <c r="D98" s="5">
+        <v>67116</v>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>OCHRE FURNITURE (NAGPUR)</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>OCHRE FURNITURE (NAGPUR)</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>NAGPUR</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>ARCO LOGISTIC</t>
+        </is>
+      </c>
+      <c r="I98" s="5"/>
+      <c r="J98" s="9"/>
     </row>
     <row r="99" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="7"/>

</xml_diff>